<commit_message>
Daily slate 2026-05-14 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-12.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-12.xlsx
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="E10" t="n">
         <v>291</v>
       </c>
       <c r="F10" t="n">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="G10" t="n">
-        <v>66.40000000000001</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="11">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2182</v>
+        <v>2189</v>
       </c>
       <c r="E17" t="n">
         <v>464</v>
       </c>
       <c r="F17" t="n">
-        <v>1718</v>
+        <v>1725</v>
       </c>
       <c r="G17" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
     </row>
   </sheetData>
@@ -1462,10 +1462,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>66.40000000000001</v>
+        <v>66.09999999999999</v>
       </c>
       <c r="C7" t="n">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="D7" t="n">
         <v>60.5</v>
@@ -1504,10 +1504,10 @@
         <v>38</v>
       </c>
       <c r="P7" t="n">
-        <v>21.3</v>
+        <v>21.2</v>
       </c>
       <c r="Q7" t="n">
-        <v>2182</v>
+        <v>2189</v>
       </c>
       <c r="R7" t="n">
         <v>41.2</v>

</xml_diff>